<commit_message>
Added 2025 NHL Predict the Pick results
</commit_message>
<xml_diff>
--- a/data/FFN_History_data.xlsx
+++ b/data/FFN_History_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\devin\Documents\Python Scripts\FFN_History\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25823FE4-C1D2-4352-9652-C2E590F023F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2807D39-5763-479E-AA98-FA2BB5416F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2831" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2840" uniqueCount="136">
   <si>
     <t>Double</t>
   </si>
@@ -80462,19 +80462,19 @@
     </row>
     <row r="823" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A823" s="9">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="B823" s="10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C823" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D823" s="9">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E823" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F823" s="9">
         <v>1</v>
@@ -80497,19 +80497,19 @@
     </row>
     <row r="824" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A824" s="9">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B824" s="10" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C824" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D824" s="9">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E824" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F824" s="9">
         <v>2</v>
@@ -80532,19 +80532,19 @@
     </row>
     <row r="825" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A825" s="9">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B825" s="10" t="s">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="C825" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D825" s="9">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E825" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F825" s="9">
         <v>3</v>
@@ -80567,10 +80567,10 @@
     </row>
     <row r="826" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A826" s="9">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="B826" s="10" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C826" s="10" t="s">
         <v>119</v>
@@ -80582,7 +80582,7 @@
         <v>1</v>
       </c>
       <c r="F826" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G826" s="10" t="s">
         <v>88</v>
@@ -80602,10 +80602,10 @@
     </row>
     <row r="827" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A827" s="9">
-        <v>164</v>
+        <v>102</v>
       </c>
       <c r="B827" s="10" t="s">
-        <v>58</v>
+        <v>5</v>
       </c>
       <c r="C827" s="10" t="s">
         <v>119</v>
@@ -80617,7 +80617,7 @@
         <v>1</v>
       </c>
       <c r="F827" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G827" s="10" t="s">
         <v>88</v>
@@ -80637,10 +80637,10 @@
     </row>
     <row r="828" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A828" s="9">
-        <v>159</v>
+        <v>125</v>
       </c>
       <c r="B828" s="10" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C828" s="10" t="s">
         <v>119</v>
@@ -80652,7 +80652,7 @@
         <v>1</v>
       </c>
       <c r="F828" s="9">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G828" s="10" t="s">
         <v>88</v>
@@ -80672,22 +80672,22 @@
     </row>
     <row r="829" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A829" s="9">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B829" s="10" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C829" s="10" t="s">
         <v>119</v>
       </c>
       <c r="D829" s="9">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="E829" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F829" s="9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G829" s="10" t="s">
         <v>88</v>
@@ -80707,22 +80707,22 @@
     </row>
     <row r="830" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A830" s="9">
-        <v>114</v>
+        <v>164</v>
       </c>
       <c r="B830" s="10" t="s">
-        <v>7</v>
+        <v>58</v>
       </c>
       <c r="C830" s="10" t="s">
         <v>119</v>
       </c>
       <c r="D830" s="9">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="E830" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F830" s="9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G830" s="10" t="s">
         <v>88</v>
@@ -80742,22 +80742,22 @@
     </row>
     <row r="831" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A831" s="9">
-        <v>125</v>
+        <v>159</v>
       </c>
       <c r="B831" s="10" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C831" s="10" t="s">
         <v>119</v>
       </c>
       <c r="D831" s="9">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="E831" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F831" s="9">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G831" s="10" t="s">
         <v>88</v>
@@ -80777,10 +80777,10 @@
     </row>
     <row r="832" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A832" s="9">
-        <v>183</v>
+        <v>102</v>
       </c>
       <c r="B832" s="10" t="s">
-        <v>116</v>
+        <v>5</v>
       </c>
       <c r="C832" s="10" t="s">
         <v>119</v>
@@ -80792,7 +80792,7 @@
         <v>2</v>
       </c>
       <c r="F832" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G832" s="10" t="s">
         <v>88</v>
@@ -80812,10 +80812,10 @@
     </row>
     <row r="833" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A833" s="9">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="B833" s="10" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C833" s="10" t="s">
         <v>119</v>
@@ -80827,7 +80827,7 @@
         <v>2</v>
       </c>
       <c r="F833" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G833" s="10" t="s">
         <v>88</v>
@@ -80847,10 +80847,10 @@
     </row>
     <row r="834" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A834" s="9">
-        <v>159</v>
+        <v>125</v>
       </c>
       <c r="B834" s="10" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C834" s="10" t="s">
         <v>119</v>
@@ -80862,7 +80862,7 @@
         <v>2</v>
       </c>
       <c r="F834" s="9">
-        <v>6.5</v>
+        <v>3</v>
       </c>
       <c r="G834" s="10" t="s">
         <v>88</v>
@@ -80882,10 +80882,10 @@
     </row>
     <row r="835" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A835" s="9">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="B835" s="10" t="s">
-        <v>65</v>
+        <v>116</v>
       </c>
       <c r="C835" s="10" t="s">
         <v>119</v>
@@ -80897,7 +80897,7 @@
         <v>2</v>
       </c>
       <c r="F835" s="9">
-        <v>6.5</v>
+        <v>4</v>
       </c>
       <c r="G835" s="10" t="s">
         <v>88</v>
@@ -80917,25 +80917,25 @@
     </row>
     <row r="836" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A836" s="9">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B836" s="10" t="s">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="C836" s="10" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="D836" s="9">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E836" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F836" s="9">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G836" s="10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H836" s="9">
         <v>1</v>
@@ -80952,25 +80952,25 @@
     </row>
     <row r="837" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A837" s="9">
-        <v>125</v>
+        <v>159</v>
       </c>
       <c r="B837" s="10" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="C837" s="10" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="D837" s="9">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E837" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F837" s="9">
-        <v>2.5</v>
+        <v>6.5</v>
       </c>
       <c r="G837" s="10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H837" s="9">
         <v>1</v>
@@ -80987,25 +80987,25 @@
     </row>
     <row r="838" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A838" s="9">
-        <v>102</v>
+        <v>173</v>
       </c>
       <c r="B838" s="10" t="s">
-        <v>5</v>
+        <v>65</v>
       </c>
       <c r="C838" s="10" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="D838" s="9">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E838" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F838" s="9">
-        <v>2.5</v>
+        <v>6.5</v>
       </c>
       <c r="G838" s="10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H838" s="9">
         <v>1</v>
@@ -81022,10 +81022,10 @@
     </row>
     <row r="839" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A839" s="9">
-        <v>123</v>
+        <v>104</v>
       </c>
       <c r="B839" s="10" t="s">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="C839" s="10" t="s">
         <v>124</v>
@@ -81037,7 +81037,7 @@
         <v>1</v>
       </c>
       <c r="F839" s="9">
-        <v>5.5</v>
+        <v>1</v>
       </c>
       <c r="G839" s="10" t="s">
         <v>86</v>
@@ -81057,10 +81057,10 @@
     </row>
     <row r="840" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A840" s="9">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="B840" s="10" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C840" s="10" t="s">
         <v>124</v>
@@ -81072,7 +81072,7 @@
         <v>1</v>
       </c>
       <c r="F840" s="9">
-        <v>5.5</v>
+        <v>2.5</v>
       </c>
       <c r="G840" s="10" t="s">
         <v>86</v>
@@ -81092,10 +81092,10 @@
     </row>
     <row r="841" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A841" s="9">
-        <v>163</v>
+        <v>102</v>
       </c>
       <c r="B841" s="10" t="s">
-        <v>57</v>
+        <v>5</v>
       </c>
       <c r="C841" s="10" t="s">
         <v>124</v>
@@ -81107,7 +81107,7 @@
         <v>1</v>
       </c>
       <c r="F841" s="9">
-        <v>5.5</v>
+        <v>2.5</v>
       </c>
       <c r="G841" s="10" t="s">
         <v>86</v>
@@ -81127,10 +81127,10 @@
     </row>
     <row r="842" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A842" s="9">
-        <v>162</v>
+        <v>123</v>
       </c>
       <c r="B842" s="10" t="s">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="C842" s="10" t="s">
         <v>124</v>
@@ -81162,10 +81162,10 @@
     </row>
     <row r="843" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A843" s="9">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B843" s="10" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C843" s="10" t="s">
         <v>124</v>
@@ -81177,7 +81177,7 @@
         <v>1</v>
       </c>
       <c r="F843" s="9">
-        <v>10.5</v>
+        <v>5.5</v>
       </c>
       <c r="G843" s="10" t="s">
         <v>86</v>
@@ -81197,10 +81197,10 @@
     </row>
     <row r="844" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A844" s="9">
-        <v>124</v>
+        <v>163</v>
       </c>
       <c r="B844" s="10" t="s">
-        <v>15</v>
+        <v>57</v>
       </c>
       <c r="C844" s="10" t="s">
         <v>124</v>
@@ -81212,7 +81212,7 @@
         <v>1</v>
       </c>
       <c r="F844" s="9">
-        <v>10.5</v>
+        <v>5.5</v>
       </c>
       <c r="G844" s="10" t="s">
         <v>86</v>
@@ -81232,10 +81232,10 @@
     </row>
     <row r="845" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A845" s="9">
-        <v>105</v>
+        <v>162</v>
       </c>
       <c r="B845" s="10" t="s">
-        <v>12</v>
+        <v>56</v>
       </c>
       <c r="C845" s="10" t="s">
         <v>124</v>
@@ -81247,7 +81247,7 @@
         <v>1</v>
       </c>
       <c r="F845" s="9">
-        <v>10.5</v>
+        <v>5.5</v>
       </c>
       <c r="G845" s="10" t="s">
         <v>86</v>
@@ -81267,10 +81267,10 @@
     </row>
     <row r="846" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A846" s="9">
-        <v>159</v>
+        <v>109</v>
       </c>
       <c r="B846" s="10" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="C846" s="10" t="s">
         <v>124</v>
@@ -81302,10 +81302,10 @@
     </row>
     <row r="847" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A847" s="9">
-        <v>106</v>
+        <v>124</v>
       </c>
       <c r="B847" s="10" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="C847" s="10" t="s">
         <v>124</v>
@@ -81337,10 +81337,10 @@
     </row>
     <row r="848" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A848" s="9">
-        <v>179</v>
+        <v>105</v>
       </c>
       <c r="B848" s="10" t="s">
-        <v>71</v>
+        <v>12</v>
       </c>
       <c r="C848" s="10" t="s">
         <v>124</v>
@@ -81372,10 +81372,10 @@
     </row>
     <row r="849" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A849" s="9">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B849" s="10" t="s">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="C849" s="10" t="s">
         <v>124</v>
@@ -81387,7 +81387,7 @@
         <v>1</v>
       </c>
       <c r="F849" s="9">
-        <v>14.5</v>
+        <v>10.5</v>
       </c>
       <c r="G849" s="10" t="s">
         <v>86</v>
@@ -81407,10 +81407,10 @@
     </row>
     <row r="850" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A850" s="9">
-        <v>186</v>
+        <v>106</v>
       </c>
       <c r="B850" s="10" t="s">
-        <v>125</v>
+        <v>3</v>
       </c>
       <c r="C850" s="10" t="s">
         <v>124</v>
@@ -81422,7 +81422,7 @@
         <v>1</v>
       </c>
       <c r="F850" s="9">
-        <v>14.5</v>
+        <v>10.5</v>
       </c>
       <c r="G850" s="10" t="s">
         <v>86</v>
@@ -81442,10 +81442,10 @@
     </row>
     <row r="851" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A851" s="9">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B851" s="10" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C851" s="10" t="s">
         <v>124</v>
@@ -81457,7 +81457,7 @@
         <v>1</v>
       </c>
       <c r="F851" s="9">
-        <v>16</v>
+        <v>10.5</v>
       </c>
       <c r="G851" s="10" t="s">
         <v>86</v>
@@ -81477,13 +81477,13 @@
     </row>
     <row r="852" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A852" s="9">
-        <v>184</v>
+        <v>164</v>
       </c>
       <c r="B852" s="10" t="s">
-        <v>122</v>
+        <v>58</v>
       </c>
       <c r="C852" s="10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D852" s="9">
         <v>2024</v>
@@ -81492,7 +81492,7 @@
         <v>1</v>
       </c>
       <c r="F852" s="9">
-        <v>1</v>
+        <v>14.5</v>
       </c>
       <c r="G852" s="10" t="s">
         <v>86</v>
@@ -81512,13 +81512,13 @@
     </row>
     <row r="853" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A853" s="9">
-        <v>102</v>
+        <v>186</v>
       </c>
       <c r="B853" s="10" t="s">
-        <v>5</v>
+        <v>125</v>
       </c>
       <c r="C853" s="10" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D853" s="9">
         <v>2024</v>
@@ -81527,7 +81527,7 @@
         <v>1</v>
       </c>
       <c r="F853" s="9">
-        <v>2</v>
+        <v>14.5</v>
       </c>
       <c r="G853" s="10" t="s">
         <v>86</v>
@@ -81547,13 +81547,13 @@
     </row>
     <row r="854" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A854" s="9">
+        <v>178</v>
+      </c>
+      <c r="B854" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="C854" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="B854" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="C854" s="10" t="s">
-        <v>126</v>
       </c>
       <c r="D854" s="9">
         <v>2024</v>
@@ -81562,7 +81562,7 @@
         <v>1</v>
       </c>
       <c r="F854" s="9">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="G854" s="10" t="s">
         <v>86</v>
@@ -81582,10 +81582,10 @@
     </row>
     <row r="855" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A855" s="9">
-        <v>164</v>
+        <v>184</v>
       </c>
       <c r="B855" s="10" t="s">
-        <v>58</v>
+        <v>122</v>
       </c>
       <c r="C855" s="10" t="s">
         <v>126</v>
@@ -81597,7 +81597,7 @@
         <v>1</v>
       </c>
       <c r="F855" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G855" s="10" t="s">
         <v>86</v>
@@ -81617,10 +81617,10 @@
     </row>
     <row r="856" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A856" s="9">
-        <v>159</v>
+        <v>102</v>
       </c>
       <c r="B856" s="10" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C856" s="10" t="s">
         <v>126</v>
@@ -81632,7 +81632,7 @@
         <v>1</v>
       </c>
       <c r="F856" s="9">
-        <v>5.5</v>
+        <v>2</v>
       </c>
       <c r="G856" s="10" t="s">
         <v>86</v>
@@ -81652,10 +81652,10 @@
     </row>
     <row r="857" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A857" s="9">
-        <v>105</v>
+        <v>124</v>
       </c>
       <c r="B857" s="10" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C857" s="10" t="s">
         <v>126</v>
@@ -81667,7 +81667,7 @@
         <v>1</v>
       </c>
       <c r="F857" s="9">
-        <v>5.5</v>
+        <v>3</v>
       </c>
       <c r="G857" s="10" t="s">
         <v>86</v>
@@ -81687,10 +81687,10 @@
     </row>
     <row r="858" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A858" s="9">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B858" s="10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C858" s="10" t="s">
         <v>126</v>
@@ -81702,7 +81702,7 @@
         <v>1</v>
       </c>
       <c r="F858" s="9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G858" s="10" t="s">
         <v>86</v>
@@ -81722,10 +81722,10 @@
     </row>
     <row r="859" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A859" s="9">
-        <v>106</v>
+        <v>159</v>
       </c>
       <c r="B859" s="10" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="C859" s="10" t="s">
         <v>126</v>
@@ -81737,7 +81737,7 @@
         <v>1</v>
       </c>
       <c r="F859" s="9">
-        <v>8.5</v>
+        <v>5.5</v>
       </c>
       <c r="G859" s="10" t="s">
         <v>86</v>
@@ -81757,10 +81757,10 @@
     </row>
     <row r="860" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A860" s="9">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="B860" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C860" s="10" t="s">
         <v>126</v>
@@ -81772,7 +81772,7 @@
         <v>1</v>
       </c>
       <c r="F860" s="9">
-        <v>8.5</v>
+        <v>5.5</v>
       </c>
       <c r="G860" s="10" t="s">
         <v>86</v>
@@ -81792,10 +81792,10 @@
     </row>
     <row r="861" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A861" s="9">
-        <v>186</v>
+        <v>162</v>
       </c>
       <c r="B861" s="10" t="s">
-        <v>125</v>
+        <v>56</v>
       </c>
       <c r="C861" s="10" t="s">
         <v>126</v>
@@ -81807,7 +81807,7 @@
         <v>1</v>
       </c>
       <c r="F861" s="9">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G861" s="10" t="s">
         <v>86</v>
@@ -81827,10 +81827,10 @@
     </row>
     <row r="862" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A862" s="9">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B862" s="10" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C862" s="10" t="s">
         <v>126</v>
@@ -81842,7 +81842,7 @@
         <v>1</v>
       </c>
       <c r="F862" s="9">
-        <v>11.5</v>
+        <v>8.5</v>
       </c>
       <c r="G862" s="10" t="s">
         <v>86</v>
@@ -81862,10 +81862,10 @@
     </row>
     <row r="863" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A863" s="9">
-        <v>163</v>
+        <v>123</v>
       </c>
       <c r="B863" s="10" t="s">
-        <v>57</v>
+        <v>13</v>
       </c>
       <c r="C863" s="10" t="s">
         <v>126</v>
@@ -81877,7 +81877,7 @@
         <v>1</v>
       </c>
       <c r="F863" s="9">
-        <v>11.5</v>
+        <v>8.5</v>
       </c>
       <c r="G863" s="10" t="s">
         <v>86</v>
@@ -81897,10 +81897,10 @@
     </row>
     <row r="864" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A864" s="9">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B864" s="10" t="s">
-        <v>71</v>
+        <v>125</v>
       </c>
       <c r="C864" s="10" t="s">
         <v>126</v>
@@ -81912,7 +81912,7 @@
         <v>1</v>
       </c>
       <c r="F864" s="9">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="G864" s="10" t="s">
         <v>86</v>
@@ -81932,13 +81932,13 @@
     </row>
     <row r="865" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A865" s="9">
-        <v>159</v>
+        <v>104</v>
       </c>
       <c r="B865" s="10" t="s">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="C865" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D865" s="9">
         <v>2024</v>
@@ -81947,7 +81947,7 @@
         <v>1</v>
       </c>
       <c r="F865" s="9">
-        <v>1</v>
+        <v>11.5</v>
       </c>
       <c r="G865" s="10" t="s">
         <v>86</v>
@@ -81967,13 +81967,13 @@
     </row>
     <row r="866" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A866" s="9">
-        <v>105</v>
+        <v>163</v>
       </c>
       <c r="B866" s="10" t="s">
-        <v>12</v>
+        <v>57</v>
       </c>
       <c r="C866" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D866" s="9">
         <v>2024</v>
@@ -81982,7 +81982,7 @@
         <v>1</v>
       </c>
       <c r="F866" s="9">
-        <v>2</v>
+        <v>11.5</v>
       </c>
       <c r="G866" s="10" t="s">
         <v>86</v>
@@ -82002,13 +82002,13 @@
     </row>
     <row r="867" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A867" s="9">
-        <v>104</v>
+        <v>179</v>
       </c>
       <c r="B867" s="10" t="s">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="C867" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D867" s="9">
         <v>2024</v>
@@ -82017,7 +82017,7 @@
         <v>1</v>
       </c>
       <c r="F867" s="9">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="G867" s="10" t="s">
         <v>86</v>
@@ -82037,10 +82037,10 @@
     </row>
     <row r="868" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A868" s="9">
-        <v>123</v>
+        <v>159</v>
       </c>
       <c r="B868" s="10" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C868" s="10" t="s">
         <v>127</v>
@@ -82052,7 +82052,7 @@
         <v>1</v>
       </c>
       <c r="F868" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G868" s="10" t="s">
         <v>86</v>
@@ -82072,10 +82072,10 @@
     </row>
     <row r="869" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A869" s="9">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B869" s="10" t="s">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="C869" s="10" t="s">
         <v>127</v>
@@ -82087,7 +82087,7 @@
         <v>1</v>
       </c>
       <c r="F869" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G869" s="10" t="s">
         <v>86</v>
@@ -82107,10 +82107,10 @@
     </row>
     <row r="870" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A870" s="9">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="B870" s="10" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="C870" s="10" t="s">
         <v>127</v>
@@ -82122,7 +82122,7 @@
         <v>1</v>
       </c>
       <c r="F870" s="9">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G870" s="10" t="s">
         <v>86</v>
@@ -82142,10 +82142,10 @@
     </row>
     <row r="871" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A871" s="9">
-        <v>102</v>
+        <v>123</v>
       </c>
       <c r="B871" s="10" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C871" s="10" t="s">
         <v>127</v>
@@ -82157,7 +82157,7 @@
         <v>1</v>
       </c>
       <c r="F871" s="9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G871" s="10" t="s">
         <v>86</v>
@@ -82177,10 +82177,10 @@
     </row>
     <row r="872" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A872" s="9">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="B872" s="10" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="C872" s="10" t="s">
         <v>127</v>
@@ -82192,7 +82192,7 @@
         <v>1</v>
       </c>
       <c r="F872" s="9">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G872" s="10" t="s">
         <v>86</v>
@@ -82212,13 +82212,13 @@
     </row>
     <row r="873" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A873" s="9">
-        <v>102</v>
+        <v>114</v>
       </c>
       <c r="B873" s="10" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C873" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D873" s="9">
         <v>2024</v>
@@ -82227,16 +82227,16 @@
         <v>1</v>
       </c>
       <c r="F873" s="9">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G873" s="10" t="s">
         <v>86</v>
       </c>
       <c r="H873" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I873" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J873" s="9">
         <v>0</v>
@@ -82247,13 +82247,13 @@
     </row>
     <row r="874" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A874" s="9">
-        <v>159</v>
+        <v>102</v>
       </c>
       <c r="B874" s="10" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="C874" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D874" s="9">
         <v>2024</v>
@@ -82262,16 +82262,16 @@
         <v>1</v>
       </c>
       <c r="F874" s="9">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G874" s="10" t="s">
         <v>86</v>
       </c>
       <c r="H874" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I874" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J874" s="9">
         <v>0</v>
@@ -82282,13 +82282,13 @@
     </row>
     <row r="875" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A875" s="9">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B875" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C875" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D875" s="9">
         <v>2024</v>
@@ -82297,16 +82297,16 @@
         <v>1</v>
       </c>
       <c r="F875" s="9">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G875" s="10" t="s">
         <v>86</v>
       </c>
       <c r="H875" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I875" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J875" s="9">
         <v>0</v>
@@ -82317,10 +82317,10 @@
     </row>
     <row r="876" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A876" s="9">
-        <v>164</v>
+        <v>102</v>
       </c>
       <c r="B876" s="10" t="s">
-        <v>58</v>
+        <v>5</v>
       </c>
       <c r="C876" s="10" t="s">
         <v>128</v>
@@ -82332,7 +82332,7 @@
         <v>1</v>
       </c>
       <c r="F876" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G876" s="10" t="s">
         <v>86</v>
@@ -82352,10 +82352,10 @@
     </row>
     <row r="877" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A877" s="9">
-        <v>106</v>
+        <v>159</v>
       </c>
       <c r="B877" s="10" t="s">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="C877" s="10" t="s">
         <v>128</v>
@@ -82367,7 +82367,7 @@
         <v>1</v>
       </c>
       <c r="F877" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G877" s="10" t="s">
         <v>86</v>
@@ -82387,10 +82387,10 @@
     </row>
     <row r="878" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A878" s="9">
-        <v>162</v>
+        <v>123</v>
       </c>
       <c r="B878" s="10" t="s">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="C878" s="10" t="s">
         <v>128</v>
@@ -82402,7 +82402,7 @@
         <v>1</v>
       </c>
       <c r="F878" s="9">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G878" s="10" t="s">
         <v>86</v>
@@ -82422,10 +82422,10 @@
     </row>
     <row r="879" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A879" s="9">
-        <v>104</v>
+        <v>164</v>
       </c>
       <c r="B879" s="10" t="s">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="C879" s="10" t="s">
         <v>128</v>
@@ -82437,7 +82437,7 @@
         <v>1</v>
       </c>
       <c r="F879" s="9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G879" s="10" t="s">
         <v>86</v>
@@ -82457,10 +82457,10 @@
     </row>
     <row r="880" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A880" s="9">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B880" s="10" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C880" s="10" t="s">
         <v>128</v>
@@ -82472,7 +82472,7 @@
         <v>1</v>
       </c>
       <c r="F880" s="9">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G880" s="10" t="s">
         <v>86</v>
@@ -82492,10 +82492,10 @@
     </row>
     <row r="881" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A881" s="9">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B881" s="10" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C881" s="10" t="s">
         <v>128</v>
@@ -82507,7 +82507,7 @@
         <v>1</v>
       </c>
       <c r="F881" s="9">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G881" s="10" t="s">
         <v>86</v>
@@ -82527,10 +82527,10 @@
     </row>
     <row r="882" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A882" s="9">
-        <v>124</v>
+        <v>104</v>
       </c>
       <c r="B882" s="10" t="s">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="C882" s="10" t="s">
         <v>128</v>
@@ -82542,7 +82542,7 @@
         <v>1</v>
       </c>
       <c r="F882" s="9">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G882" s="10" t="s">
         <v>86</v>
@@ -82562,10 +82562,10 @@
     </row>
     <row r="883" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A883" s="9">
-        <v>167</v>
+        <v>109</v>
       </c>
       <c r="B883" s="10" t="s">
-        <v>60</v>
+        <v>2</v>
       </c>
       <c r="C883" s="10" t="s">
         <v>128</v>
@@ -82577,7 +82577,7 @@
         <v>1</v>
       </c>
       <c r="F883" s="9">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G883" s="10" t="s">
         <v>86</v>
@@ -82597,10 +82597,10 @@
     </row>
     <row r="884" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A884" s="9">
-        <v>114</v>
+        <v>156</v>
       </c>
       <c r="B884" s="10" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
       <c r="C884" s="10" t="s">
         <v>128</v>
@@ -82612,7 +82612,7 @@
         <v>1</v>
       </c>
       <c r="F884" s="9">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G884" s="10" t="s">
         <v>86</v>
@@ -82632,13 +82632,13 @@
     </row>
     <row r="885" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A885" s="9">
-        <v>102</v>
+        <v>124</v>
       </c>
       <c r="B885" s="10" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C885" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D885" s="9">
         <v>2024</v>
@@ -82647,7 +82647,7 @@
         <v>1</v>
       </c>
       <c r="F885" s="9">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G885" s="10" t="s">
         <v>86</v>
@@ -82667,13 +82667,13 @@
     </row>
     <row r="886" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A886" s="9">
-        <v>104</v>
+        <v>167</v>
       </c>
       <c r="B886" s="10" t="s">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="C886" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D886" s="9">
         <v>2024</v>
@@ -82682,7 +82682,7 @@
         <v>1</v>
       </c>
       <c r="F886" s="9">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G886" s="10" t="s">
         <v>86</v>
@@ -82702,13 +82702,13 @@
     </row>
     <row r="887" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A887" s="9">
-        <v>164</v>
+        <v>114</v>
       </c>
       <c r="B887" s="10" t="s">
-        <v>58</v>
+        <v>7</v>
       </c>
       <c r="C887" s="10" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D887" s="9">
         <v>2024</v>
@@ -82717,7 +82717,7 @@
         <v>1</v>
       </c>
       <c r="F887" s="9">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G887" s="10" t="s">
         <v>86</v>
@@ -82737,10 +82737,10 @@
     </row>
     <row r="888" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A888" s="9">
-        <v>123</v>
+        <v>102</v>
       </c>
       <c r="B888" s="10" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C888" s="10" t="s">
         <v>129</v>
@@ -82752,7 +82752,7 @@
         <v>1</v>
       </c>
       <c r="F888" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G888" s="10" t="s">
         <v>86</v>
@@ -82772,10 +82772,10 @@
     </row>
     <row r="889" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A889" s="9">
-        <v>162</v>
+        <v>104</v>
       </c>
       <c r="B889" s="10" t="s">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="C889" s="10" t="s">
         <v>129</v>
@@ -82787,7 +82787,7 @@
         <v>1</v>
       </c>
       <c r="F889" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G889" s="10" t="s">
         <v>86</v>
@@ -82807,10 +82807,10 @@
     </row>
     <row r="890" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A890" s="9">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B890" s="10" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C890" s="10" t="s">
         <v>129</v>
@@ -82822,7 +82822,7 @@
         <v>1</v>
       </c>
       <c r="F890" s="9">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G890" s="10" t="s">
         <v>86</v>
@@ -82842,10 +82842,10 @@
     </row>
     <row r="891" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A891" s="9">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="B891" s="10" t="s">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="C891" s="10" t="s">
         <v>129</v>
@@ -82857,7 +82857,7 @@
         <v>1</v>
       </c>
       <c r="F891" s="9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G891" s="10" t="s">
         <v>86</v>
@@ -82877,10 +82877,10 @@
     </row>
     <row r="892" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A892" s="9">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B892" s="10" t="s">
-        <v>14</v>
+        <v>56</v>
       </c>
       <c r="C892" s="10" t="s">
         <v>129</v>
@@ -82892,7 +82892,7 @@
         <v>1</v>
       </c>
       <c r="F892" s="9">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G892" s="10" t="s">
         <v>86</v>
@@ -82912,10 +82912,10 @@
     </row>
     <row r="893" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A893" s="9">
-        <v>106</v>
+        <v>167</v>
       </c>
       <c r="B893" s="10" t="s">
-        <v>3</v>
+        <v>60</v>
       </c>
       <c r="C893" s="10" t="s">
         <v>129</v>
@@ -82927,7 +82927,7 @@
         <v>1</v>
       </c>
       <c r="F893" s="9">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G893" s="10" t="s">
         <v>86</v>
@@ -82947,10 +82947,10 @@
     </row>
     <row r="894" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A894" s="9">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="B894" s="10" t="s">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="C894" s="10" t="s">
         <v>129</v>
@@ -82962,7 +82962,7 @@
         <v>1</v>
       </c>
       <c r="F894" s="9">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G894" s="10" t="s">
         <v>86</v>
@@ -82982,10 +82982,10 @@
     </row>
     <row r="895" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A895" s="9">
-        <v>114</v>
+        <v>159</v>
       </c>
       <c r="B895" s="10" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="C895" s="10" t="s">
         <v>129</v>
@@ -82997,7 +82997,7 @@
         <v>1</v>
       </c>
       <c r="F895" s="9">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G895" s="10" t="s">
         <v>86</v>
@@ -83017,10 +83017,10 @@
     </row>
     <row r="896" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A896" s="9">
-        <v>156</v>
+        <v>106</v>
       </c>
       <c r="B896" s="10" t="s">
-        <v>51</v>
+        <v>3</v>
       </c>
       <c r="C896" s="10" t="s">
         <v>129</v>
@@ -83032,7 +83032,7 @@
         <v>1</v>
       </c>
       <c r="F896" s="9">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="G896" s="10" t="s">
         <v>86</v>
@@ -83052,31 +83052,31 @@
     </row>
     <row r="897" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A897" s="9">
-        <v>102</v>
+        <v>124</v>
       </c>
       <c r="B897" s="10" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C897" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D897" s="9">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="E897" s="9">
         <v>1</v>
       </c>
       <c r="F897" s="9">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G897" s="10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H897" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I897" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J897" s="9">
         <v>0</v>
@@ -83087,31 +83087,31 @@
     </row>
     <row r="898" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A898" s="9">
-        <v>159</v>
+        <v>114</v>
       </c>
       <c r="B898" s="10" t="s">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="C898" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D898" s="9">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="E898" s="9">
         <v>1</v>
       </c>
       <c r="F898" s="9">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="G898" s="10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H898" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I898" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J898" s="9">
         <v>0</v>
@@ -83122,31 +83122,31 @@
     </row>
     <row r="899" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A899" s="9">
-        <v>173</v>
+        <v>156</v>
       </c>
       <c r="B899" s="10" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
       <c r="C899" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D899" s="9">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="E899" s="9">
         <v>1</v>
       </c>
       <c r="F899" s="9">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G899" s="10" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H899" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I899" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J899" s="9">
         <v>0</v>
@@ -83157,10 +83157,10 @@
     </row>
     <row r="900" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A900" s="9">
-        <v>161</v>
+        <v>102</v>
       </c>
       <c r="B900" s="10" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="C900" s="10" t="s">
         <v>130</v>
@@ -83172,7 +83172,7 @@
         <v>1</v>
       </c>
       <c r="F900" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G900" s="10" t="s">
         <v>88</v>
@@ -83192,10 +83192,10 @@
     </row>
     <row r="901" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A901" s="9">
-        <v>172</v>
+        <v>159</v>
       </c>
       <c r="B901" s="10" t="s">
-        <v>64</v>
+        <v>14</v>
       </c>
       <c r="C901" s="10" t="s">
         <v>130</v>
@@ -83207,7 +83207,7 @@
         <v>1</v>
       </c>
       <c r="F901" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G901" s="10" t="s">
         <v>88</v>
@@ -83227,10 +83227,10 @@
     </row>
     <row r="902" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A902" s="9">
-        <v>105</v>
+        <v>173</v>
       </c>
       <c r="B902" s="10" t="s">
-        <v>12</v>
+        <v>65</v>
       </c>
       <c r="C902" s="10" t="s">
         <v>130</v>
@@ -83242,7 +83242,7 @@
         <v>1</v>
       </c>
       <c r="F902" s="9">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G902" s="10" t="s">
         <v>88</v>
@@ -83262,34 +83262,34 @@
     </row>
     <row r="903" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A903" s="9">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B903" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C903" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D903" s="9">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E903" s="9">
         <v>1</v>
       </c>
       <c r="F903" s="9">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G903" s="10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H903" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I903" s="9">
         <v>0</v>
       </c>
       <c r="J903" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K903" s="9">
         <v>0</v>
@@ -83297,34 +83297,34 @@
     </row>
     <row r="904" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A904" s="9">
-        <v>105</v>
+        <v>172</v>
       </c>
       <c r="B904" s="10" t="s">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="C904" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D904" s="9">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E904" s="9">
         <v>1</v>
       </c>
       <c r="F904" s="9">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G904" s="10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H904" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I904" s="9">
         <v>0</v>
       </c>
       <c r="J904" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K904" s="9">
         <v>0</v>
@@ -83332,34 +83332,34 @@
     </row>
     <row r="905" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A905" s="9">
-        <v>124</v>
+        <v>105</v>
       </c>
       <c r="B905" s="10" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C905" s="10" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D905" s="9">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E905" s="9">
         <v>1</v>
       </c>
       <c r="F905" s="9">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G905" s="10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H905" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I905" s="9">
         <v>0</v>
       </c>
       <c r="J905" s="9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K905" s="9">
         <v>0</v>
@@ -83367,10 +83367,10 @@
     </row>
     <row r="906" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A906" s="9">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B906" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C906" s="10" t="s">
         <v>131</v>
@@ -83382,7 +83382,7 @@
         <v>1</v>
       </c>
       <c r="F906" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G906" s="10" t="s">
         <v>86</v>
@@ -83402,10 +83402,10 @@
     </row>
     <row r="907" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A907" s="9">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="B907" s="10" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C907" s="10" t="s">
         <v>131</v>
@@ -83417,7 +83417,7 @@
         <v>1</v>
       </c>
       <c r="F907" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G907" s="10" t="s">
         <v>86</v>
@@ -83437,10 +83437,10 @@
     </row>
     <row r="908" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A908" s="9">
-        <v>188</v>
+        <v>124</v>
       </c>
       <c r="B908" s="10" t="s">
-        <v>123</v>
+        <v>15</v>
       </c>
       <c r="C908" s="10" t="s">
         <v>131</v>
@@ -83452,7 +83452,7 @@
         <v>1</v>
       </c>
       <c r="F908" s="9">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G908" s="10" t="s">
         <v>86</v>
@@ -83472,10 +83472,10 @@
     </row>
     <row r="909" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A909" s="9">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B909" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C909" s="10" t="s">
         <v>131</v>
@@ -83487,7 +83487,7 @@
         <v>1</v>
       </c>
       <c r="F909" s="9">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="G909" s="10" t="s">
         <v>86</v>
@@ -83507,10 +83507,10 @@
     </row>
     <row r="910" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A910" s="9">
-        <v>123</v>
+        <v>102</v>
       </c>
       <c r="B910" s="10" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C910" s="10" t="s">
         <v>131</v>
@@ -83522,7 +83522,7 @@
         <v>1</v>
       </c>
       <c r="F910" s="9">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G910" s="10" t="s">
         <v>86</v>
@@ -83542,10 +83542,10 @@
     </row>
     <row r="911" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A911" s="9">
-        <v>156</v>
+        <v>188</v>
       </c>
       <c r="B911" s="10" t="s">
-        <v>51</v>
+        <v>123</v>
       </c>
       <c r="C911" s="10" t="s">
         <v>131</v>
@@ -83557,7 +83557,7 @@
         <v>1</v>
       </c>
       <c r="F911" s="9">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="G911" s="10" t="s">
         <v>86</v>
@@ -83577,10 +83577,10 @@
     </row>
     <row r="912" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A912" s="9">
-        <v>187</v>
+        <v>164</v>
       </c>
       <c r="B912" s="10" t="s">
-        <v>121</v>
+        <v>58</v>
       </c>
       <c r="C912" s="10" t="s">
         <v>131</v>
@@ -83592,7 +83592,7 @@
         <v>1</v>
       </c>
       <c r="F912" s="9">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="G912" s="10" t="s">
         <v>86</v>
@@ -83612,13 +83612,13 @@
     </row>
     <row r="913" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A913" s="9">
-        <v>102</v>
+        <v>123</v>
       </c>
       <c r="B913" s="10" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C913" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D913" s="9">
         <v>2024</v>
@@ -83627,7 +83627,7 @@
         <v>1</v>
       </c>
       <c r="F913" s="9">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G913" s="10" t="s">
         <v>86</v>
@@ -83647,13 +83647,13 @@
     </row>
     <row r="914" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A914" s="9">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="B914" s="10" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C914" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D914" s="9">
         <v>2024</v>
@@ -83662,7 +83662,7 @@
         <v>1</v>
       </c>
       <c r="F914" s="9">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G914" s="10" t="s">
         <v>86</v>
@@ -83682,13 +83682,13 @@
     </row>
     <row r="915" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A915" s="9">
-        <v>162</v>
+        <v>187</v>
       </c>
       <c r="B915" s="10" t="s">
-        <v>56</v>
+        <v>121</v>
       </c>
       <c r="C915" s="10" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D915" s="9">
         <v>2024</v>
@@ -83697,7 +83697,7 @@
         <v>1</v>
       </c>
       <c r="F915" s="9">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="G915" s="10" t="s">
         <v>86</v>
@@ -83717,10 +83717,10 @@
     </row>
     <row r="916" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A916" s="9">
-        <v>123</v>
+        <v>102</v>
       </c>
       <c r="B916" s="10" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C916" s="10" t="s">
         <v>132</v>
@@ -83732,7 +83732,7 @@
         <v>1</v>
       </c>
       <c r="F916" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G916" s="10" t="s">
         <v>86</v>
@@ -83752,10 +83752,10 @@
     </row>
     <row r="917" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A917" s="9">
-        <v>104</v>
+        <v>163</v>
       </c>
       <c r="B917" s="10" t="s">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="C917" s="10" t="s">
         <v>132</v>
@@ -83767,7 +83767,7 @@
         <v>1</v>
       </c>
       <c r="F917" s="9">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G917" s="10" t="s">
         <v>86</v>
@@ -83787,10 +83787,10 @@
     </row>
     <row r="918" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A918" s="9">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B918" s="10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C918" s="10" t="s">
         <v>132</v>
@@ -83802,7 +83802,7 @@
         <v>1</v>
       </c>
       <c r="F918" s="9">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G918" s="10" t="s">
         <v>86</v>
@@ -83822,10 +83822,10 @@
     </row>
     <row r="919" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A919" s="9">
-        <v>156</v>
+        <v>123</v>
       </c>
       <c r="B919" s="10" t="s">
-        <v>51</v>
+        <v>13</v>
       </c>
       <c r="C919" s="10" t="s">
         <v>132</v>
@@ -83837,7 +83837,7 @@
         <v>1</v>
       </c>
       <c r="F919" s="9">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G919" s="10" t="s">
         <v>86</v>
@@ -83857,10 +83857,10 @@
     </row>
     <row r="920" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A920" s="9">
-        <v>187</v>
+        <v>104</v>
       </c>
       <c r="B920" s="10" t="s">
-        <v>121</v>
+        <v>0</v>
       </c>
       <c r="C920" s="10" t="s">
         <v>132</v>
@@ -83872,7 +83872,7 @@
         <v>1</v>
       </c>
       <c r="F920" s="9">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="G920" s="10" t="s">
         <v>86</v>
@@ -83892,10 +83892,10 @@
     </row>
     <row r="921" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A921" s="9">
-        <v>124</v>
+        <v>164</v>
       </c>
       <c r="B921" s="10" t="s">
-        <v>15</v>
+        <v>58</v>
       </c>
       <c r="C921" s="10" t="s">
         <v>132</v>
@@ -83907,7 +83907,7 @@
         <v>1</v>
       </c>
       <c r="F921" s="9">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G921" s="10" t="s">
         <v>86</v>
@@ -83927,13 +83927,13 @@
     </row>
     <row r="922" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A922" s="9">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="B922" s="10" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C922" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D922" s="9">
         <v>2024</v>
@@ -83942,7 +83942,7 @@
         <v>1</v>
       </c>
       <c r="F922" s="9">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="G922" s="10" t="s">
         <v>86</v>
@@ -83962,13 +83962,13 @@
     </row>
     <row r="923" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A923" s="9">
-        <v>105</v>
+        <v>187</v>
       </c>
       <c r="B923" s="10" t="s">
-        <v>12</v>
+        <v>121</v>
       </c>
       <c r="C923" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D923" s="9">
         <v>2024</v>
@@ -83977,7 +83977,7 @@
         <v>1</v>
       </c>
       <c r="F923" s="9">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G923" s="10" t="s">
         <v>86</v>
@@ -83997,13 +83997,13 @@
     </row>
     <row r="924" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A924" s="9">
-        <v>102</v>
+        <v>124</v>
       </c>
       <c r="B924" s="10" t="s">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="C924" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D924" s="9">
         <v>2024</v>
@@ -84012,7 +84012,7 @@
         <v>1</v>
       </c>
       <c r="F924" s="9">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G924" s="10" t="s">
         <v>86</v>
@@ -84032,10 +84032,10 @@
     </row>
     <row r="925" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A925" s="9">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="B925" s="10" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C925" s="10" t="s">
         <v>133</v>
@@ -84047,7 +84047,7 @@
         <v>1</v>
       </c>
       <c r="F925" s="9">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G925" s="10" t="s">
         <v>86</v>
@@ -84067,10 +84067,10 @@
     </row>
     <row r="926" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A926" s="9">
-        <v>155</v>
+        <v>105</v>
       </c>
       <c r="B926" s="10" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="C926" s="10" t="s">
         <v>133</v>
@@ -84082,7 +84082,7 @@
         <v>1</v>
       </c>
       <c r="F926" s="9">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G926" s="10" t="s">
         <v>86</v>
@@ -84102,10 +84102,10 @@
     </row>
     <row r="927" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A927" s="9">
-        <v>123</v>
+        <v>102</v>
       </c>
       <c r="B927" s="10" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="C927" s="10" t="s">
         <v>133</v>
@@ -84117,7 +84117,7 @@
         <v>1</v>
       </c>
       <c r="F927" s="9">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G927" s="10" t="s">
         <v>86</v>
@@ -84137,10 +84137,10 @@
     </row>
     <row r="928" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A928" s="9">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B928" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C928" s="10" t="s">
         <v>133</v>
@@ -84152,7 +84152,7 @@
         <v>1</v>
       </c>
       <c r="F928" s="9">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G928" s="10" t="s">
         <v>86</v>
@@ -84172,10 +84172,10 @@
     </row>
     <row r="929" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A929" s="9">
-        <v>114</v>
+        <v>155</v>
       </c>
       <c r="B929" s="10" t="s">
-        <v>7</v>
+        <v>50</v>
       </c>
       <c r="C929" s="10" t="s">
         <v>133</v>
@@ -84187,7 +84187,7 @@
         <v>1</v>
       </c>
       <c r="F929" s="9">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G929" s="10" t="s">
         <v>86</v>
@@ -84205,20 +84205,110 @@
         <v>0</v>
       </c>
     </row>
-    <row r="930" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B930" s="3"/>
-      <c r="C930" s="3"/>
-      <c r="G930" s="3"/>
-    </row>
-    <row r="931" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B931" s="3"/>
-      <c r="C931" s="3"/>
-      <c r="G931" s="3"/>
-    </row>
-    <row r="932" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B932" s="3"/>
-      <c r="C932" s="3"/>
-      <c r="G932" s="3"/>
+    <row r="930" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A930" s="9">
+        <v>123</v>
+      </c>
+      <c r="B930" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="C930" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D930" s="9">
+        <v>2024</v>
+      </c>
+      <c r="E930" s="9">
+        <v>1</v>
+      </c>
+      <c r="F930" s="9">
+        <v>6</v>
+      </c>
+      <c r="G930" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="H930" s="9">
+        <v>0</v>
+      </c>
+      <c r="I930" s="9">
+        <v>0</v>
+      </c>
+      <c r="J930" s="9">
+        <v>1</v>
+      </c>
+      <c r="K930" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="931" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A931" s="9">
+        <v>173</v>
+      </c>
+      <c r="B931" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C931" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D931" s="9">
+        <v>2024</v>
+      </c>
+      <c r="E931" s="9">
+        <v>1</v>
+      </c>
+      <c r="F931" s="9">
+        <v>7</v>
+      </c>
+      <c r="G931" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="H931" s="9">
+        <v>0</v>
+      </c>
+      <c r="I931" s="9">
+        <v>0</v>
+      </c>
+      <c r="J931" s="9">
+        <v>1</v>
+      </c>
+      <c r="K931" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="932" spans="1:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A932" s="9">
+        <v>114</v>
+      </c>
+      <c r="B932" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C932" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D932" s="9">
+        <v>2024</v>
+      </c>
+      <c r="E932" s="9">
+        <v>1</v>
+      </c>
+      <c r="F932" s="9">
+        <v>8</v>
+      </c>
+      <c r="G932" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="H932" s="9">
+        <v>0</v>
+      </c>
+      <c r="I932" s="9">
+        <v>0</v>
+      </c>
+      <c r="J932" s="9">
+        <v>1</v>
+      </c>
+      <c r="K932" s="9">
+        <v>0</v>
+      </c>
     </row>
     <row r="933" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
       <c r="B933" s="3"/>

</xml_diff>